<commit_message>
Edit: 177808641339 - Chanel Classic Flap Maxi
</commit_message>
<xml_diff>
--- a/edited.xlsx
+++ b/edited.xlsx
@@ -58,9 +58,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,9 +424,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Backfill: items 1-10 already edited
</commit_message>
<xml_diff>
--- a/edited.xlsx
+++ b/edited.xlsx
@@ -424,13 +424,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1"/>
     <row r="2"/>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix: rebuild edited.xlsx with headers + all 11 edited items
</commit_message>
<xml_diff>
--- a/edited.xlsx
+++ b/edited.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="edited" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="edited" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -424,36 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1"/>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:BB1"/>
+  <dimension ref="A1:BB12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -784,6 +754,1267 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>178027307182</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>FENDI Baguette Charm Crossbody Bag Nano 7AR844</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>USD 440.64</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Pre-owned - Good</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Some signs of use, but well-maintained and in good condition</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Fendi</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>7AR844</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178027307182</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Fendi</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Crossbody</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Mixed Materials</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>Fendi Baguette</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>7AR844</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>Nano</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>messenger_bag_type</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>177800599413</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BOTTEGA VENETA Cassette Calfskin Belt Mini New Sage</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>USD 716.00</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Pre-owned - Fair</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Shows signs of use, but is in good condition having been lovingly cared for.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Bottega Veneta</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/177800599413</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Bottega Veneta</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Crossbody</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Leather</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>Leather</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>Bottega Veneta Cassette</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>Leather</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>Mini</t>
+        </is>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>non_english:conditionDescription</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>178027307184</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GUCCI Paddle Lock Chain Shoulder Bag Large 409486</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>USD 689.12</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Pre-owned - Excellent</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Noticeable signs of use, but carefully maintained</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>409486</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178027307184</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Shoulder Bag</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Multicolor</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>Canvas</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Gucci GG</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Lock</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>409486</t>
+        </is>
+      </c>
+      <c r="BB4" t="inlineStr">
+        <is>
+          <t>messenger_bag_type</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>178026165564</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>LOUIS VUITTON Side Trunk Monogram Canvas Shoulder Bag MM M46358</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>USD 2712.58</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Pre-owned - Excellent</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Some signs of use, but well-maintained and in good condition</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>LOUIS VUITTON</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178026165564</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>LOUIS VUITTON</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Messenger Bags</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Messenger Bags</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Multicolor</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>Canvas</t>
+        </is>
+      </c>
+      <c r="BB5" t="inlineStr">
+        <is>
+          <t>messenger_bag_type</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>178045045338</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PRADA Pocono Stud Bucket Bag 1BE027</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>USD 610.91</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Pre-owned - Good</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Some signs of use, but well-maintained and in good condition</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>PRADA</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>1BE027</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178045045338</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>PRADA</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Bucket &amp; Drawstring Bag</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Nylon</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>Drawstring</t>
+        </is>
+      </c>
+      <c r="AG6" t="inlineStr">
+        <is>
+          <t>PRADA Pocono</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AL6" t="inlineStr">
+        <is>
+          <t>1BE027</t>
+        </is>
+      </c>
+      <c r="BB6" t="inlineStr">
+        <is>
+          <t>messenger_bag_type</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>178047195067</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PRADA Giallo Tessuto Chain Flap Bag 1BD199</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>USD 415.41</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Pre-owned - Good</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Some signs of use, but well-maintained and in good condition</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>PRADA</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>1BD199</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178047195067</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>PRADA</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Shoulder Bag</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>Nylon</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>PRADA Tessuto</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>1BD199</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>messenger_bag_type, non_english:aspect_Exterior Color</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>178008164473</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GUCCI x Adidas Shoulder Bag 702427</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>USD 701.18</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Pre-owned - Excellent</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Noticeable signs of use, but carefully maintained</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>702427</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178008164473</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Shoulder Bag</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Canvas, Leather</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>Detachable Strap</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>702427</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>messenger_bag_type, non_english:aspect_Exterior Color|description</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>178032429937</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PRADA Galleria Piano Shoulder Bag Large 1BA274</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>USD 567.27</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Pre-owned - Good</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Some signs of use, but well-maintained and in good condition</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>PRADA</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>1BA274</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178032429937</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>PRADA</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Shoulder Bag</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Navy</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Leather</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>Prada Galleria</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>Saffiano</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>PRADA Galleria</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>1BA274</t>
+        </is>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>messenger_bag_type, non_english:aspect_Exterior Color</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>178047621011</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PRADA Panier Saffiano Bucket Bag 1BA217</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>USD 1110.14</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Pre-owned - Good</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Some signs of use, but well-maintained and in good condition</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>PRADA</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>1BA217</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178047621011</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>PRADA</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Bucket &amp; Drawstring Bag</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Off-White</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>Leather</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>PRADA Panier</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>Saffiano</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>PRADA Panier</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>1BA217</t>
+        </is>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>messenger_bag_type, non_english:title|aspect_Exterior Color</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>178047404048</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>GUCCI x Adidas Shoulder Bag Small 702427</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>USD 765.06</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Pre-owned - Good</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Some signs of use, but well-maintained and in good condition</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>702427</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>1</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178047404048</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Shoulder Bag</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Leather</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>702427</t>
+        </is>
+      </c>
+      <c r="BB11" t="inlineStr">
+        <is>
+          <t>messenger_bag_type, non_english:aspect_Exterior Color</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>177808641339</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Chanel Classic Flap Maxi Quilted Lambskin Gold Chain Shoulder Bag</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>USD 3627.89</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Pre-owned - Fair</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Good condition for daily use with noticeable signs of use.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>CHANEL</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/177808641339</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>CHANEL</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Shoulder Bag</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Beige</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>Leather</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>13 in</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Argyle/Diamond</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>Rectangle</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>Turn Lock</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>9 in</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>Lambskin</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>4 in</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>Original Dust Bag</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>Chanel Classic</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>Quilted</t>
+        </is>
+      </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>CHANEL Classic Flap</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr"/>
+      <c r="AN12" t="inlineStr"/>
+      <c r="AO12" t="inlineStr"/>
+      <c r="AP12" t="inlineStr"/>
+      <c r="AQ12" t="inlineStr"/>
+      <c r="AR12" t="inlineStr"/>
+      <c r="AS12" t="inlineStr"/>
+      <c r="AT12" t="inlineStr"/>
+      <c r="AU12" t="inlineStr"/>
+      <c r="AV12" t="inlineStr"/>
+      <c r="AW12" t="inlineStr"/>
+      <c r="AX12" t="inlineStr"/>
+      <c r="AY12" t="inlineStr"/>
+      <c r="AZ12" t="inlineStr"/>
+      <c r="BA12" t="inlineStr"/>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>non_english:conditionDescription</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Edit: 178047621207 - GUCCI Holsbit 1955 Mini Bag
</commit_message>
<xml_diff>
--- a/edited.xlsx
+++ b/edited.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB12"/>
+  <dimension ref="A1:BB13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1845,7 +1845,6 @@
           <t>USD 3627.89</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>Pre-owned - Fair</t>
@@ -1871,8 +1870,6 @@
           <t>CHANEL</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
         <v>1</v>
       </c>
@@ -1896,7 +1893,6 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr">
         <is>
           <t>Shoulder Bag</t>
@@ -1912,7 +1908,6 @@
           <t>Leather</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr"/>
       <c r="V12" t="inlineStr">
         <is>
           <t>13 in</t>
@@ -1993,25 +1988,151 @@
           <t>CHANEL Classic Flap</t>
         </is>
       </c>
-      <c r="AL12" t="inlineStr"/>
-      <c r="AM12" t="inlineStr"/>
-      <c r="AN12" t="inlineStr"/>
-      <c r="AO12" t="inlineStr"/>
-      <c r="AP12" t="inlineStr"/>
-      <c r="AQ12" t="inlineStr"/>
-      <c r="AR12" t="inlineStr"/>
-      <c r="AS12" t="inlineStr"/>
-      <c r="AT12" t="inlineStr"/>
-      <c r="AU12" t="inlineStr"/>
-      <c r="AV12" t="inlineStr"/>
-      <c r="AW12" t="inlineStr"/>
-      <c r="AX12" t="inlineStr"/>
-      <c r="AY12" t="inlineStr"/>
-      <c r="AZ12" t="inlineStr"/>
-      <c r="BA12" t="inlineStr"/>
       <c r="BB12" t="inlineStr">
         <is>
           <t>non_english:conditionDescription</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>178047621207</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>GUCCI Holsbit 1955 Mini Bag Brown 625615</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>USD 616.94</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Pre-owned - Good</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Some signs of use, but well-maintained and in good condition</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178047621207</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Crossbody</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>Leather</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
+      <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
+      <c r="AC13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr"/>
+      <c r="AE13" t="inlineStr"/>
+      <c r="AF13" t="inlineStr"/>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>GUCCI Holsbit</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>Gucci Horsebit 1955</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr"/>
+      <c r="AM13" t="inlineStr"/>
+      <c r="AN13" t="inlineStr"/>
+      <c r="AO13" t="inlineStr"/>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>Leather</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr"/>
+      <c r="AR13" t="inlineStr"/>
+      <c r="AS13" t="inlineStr"/>
+      <c r="AT13" t="inlineStr"/>
+      <c r="AU13" t="inlineStr"/>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>Mini</t>
+        </is>
+      </c>
+      <c r="AW13" t="inlineStr"/>
+      <c r="AX13" t="inlineStr"/>
+      <c r="AY13" t="inlineStr"/>
+      <c r="AZ13" t="inlineStr"/>
+      <c r="BA13" t="inlineStr"/>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>messenger_bag_type, non_english:aspect_Exterior Color</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Edit: 178047621211 - BALENCIAGA Classic Town Motor Bag
</commit_message>
<xml_diff>
--- a/edited.xlsx
+++ b/edited.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB13"/>
+  <dimension ref="A1:BB14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2010,7 +2010,6 @@
           <t>USD 616.94</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>Pre-owned - Good</t>
@@ -2036,8 +2035,6 @@
           <t>Gucci</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
         <v>1</v>
       </c>
@@ -2061,7 +2058,6 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr">
         <is>
           <t>Crossbody</t>
@@ -2077,60 +2073,158 @@
           <t>Leather</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr"/>
-      <c r="V13" t="inlineStr"/>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr"/>
-      <c r="AA13" t="inlineStr"/>
-      <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="inlineStr"/>
-      <c r="AD13" t="inlineStr"/>
-      <c r="AE13" t="inlineStr"/>
-      <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr">
         <is>
           <t>GUCCI Holsbit</t>
         </is>
       </c>
-      <c r="AH13" t="inlineStr"/>
       <c r="AI13" t="inlineStr">
         <is>
           <t>Italy</t>
         </is>
       </c>
-      <c r="AJ13" t="inlineStr"/>
       <c r="AK13" t="inlineStr">
         <is>
           <t>Gucci Horsebit 1955</t>
         </is>
       </c>
-      <c r="AL13" t="inlineStr"/>
-      <c r="AM13" t="inlineStr"/>
-      <c r="AN13" t="inlineStr"/>
-      <c r="AO13" t="inlineStr"/>
       <c r="AP13" t="inlineStr">
         <is>
           <t>Leather</t>
         </is>
       </c>
-      <c r="AQ13" t="inlineStr"/>
-      <c r="AR13" t="inlineStr"/>
-      <c r="AS13" t="inlineStr"/>
-      <c r="AT13" t="inlineStr"/>
-      <c r="AU13" t="inlineStr"/>
       <c r="AV13" t="inlineStr">
         <is>
           <t>Mini</t>
         </is>
       </c>
-      <c r="AW13" t="inlineStr"/>
-      <c r="AX13" t="inlineStr"/>
-      <c r="AY13" t="inlineStr"/>
-      <c r="AZ13" t="inlineStr"/>
-      <c r="BA13" t="inlineStr"/>
       <c r="BB13" t="inlineStr">
+        <is>
+          <t>messenger_bag_type, non_english:aspect_Exterior Color</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>178047621211</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>BALENCIAGA Classic Town Motor Bag 240579</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>USD 1001.92</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Pre-owned - Good</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Some signs of use, but well-maintained and in good condition</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>BALENCIAGA</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178047621211</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>BALENCIAGA</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Messenger Bags</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Messenger Bags</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Gray/계열</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>Leather</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
+      <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
+      <c r="Z14" t="inlineStr"/>
+      <c r="AA14" t="inlineStr"/>
+      <c r="AB14" t="inlineStr"/>
+      <c r="AC14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr"/>
+      <c r="AE14" t="inlineStr"/>
+      <c r="AF14" t="inlineStr"/>
+      <c r="AG14" t="inlineStr"/>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr"/>
+      <c r="AM14" t="inlineStr"/>
+      <c r="AN14" t="inlineStr"/>
+      <c r="AO14" t="inlineStr"/>
+      <c r="AP14" t="inlineStr"/>
+      <c r="AQ14" t="inlineStr"/>
+      <c r="AR14" t="inlineStr"/>
+      <c r="AS14" t="inlineStr"/>
+      <c r="AT14" t="inlineStr"/>
+      <c r="AU14" t="inlineStr"/>
+      <c r="AV14" t="inlineStr"/>
+      <c r="AW14" t="inlineStr"/>
+      <c r="AX14" t="inlineStr"/>
+      <c r="AY14" t="inlineStr"/>
+      <c r="AZ14" t="inlineStr"/>
+      <c r="BA14" t="inlineStr"/>
+      <c r="BB14" t="inlineStr">
         <is>
           <t>messenger_bag_type, non_english:aspect_Exterior Color</t>
         </is>

</xml_diff>

<commit_message>
Edit: 177808647882 - LV Mylockme Chain Pochette
</commit_message>
<xml_diff>
--- a/edited.xlsx
+++ b/edited.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB14"/>
+  <dimension ref="A1:BB15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2120,7 +2120,6 @@
           <t>USD 1001.92</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>Pre-owned - Good</t>
@@ -2146,8 +2145,6 @@
           <t>BALENCIAGA</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
         <v>1</v>
       </c>
@@ -2191,42 +2188,203 @@
           <t>Leather</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr"/>
-      <c r="V14" t="inlineStr"/>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
-      <c r="Z14" t="inlineStr"/>
-      <c r="AA14" t="inlineStr"/>
-      <c r="AB14" t="inlineStr"/>
-      <c r="AC14" t="inlineStr"/>
-      <c r="AD14" t="inlineStr"/>
-      <c r="AE14" t="inlineStr"/>
-      <c r="AF14" t="inlineStr"/>
-      <c r="AG14" t="inlineStr"/>
-      <c r="AH14" t="inlineStr"/>
-      <c r="AI14" t="inlineStr"/>
-      <c r="AJ14" t="inlineStr"/>
-      <c r="AK14" t="inlineStr"/>
-      <c r="AL14" t="inlineStr"/>
-      <c r="AM14" t="inlineStr"/>
-      <c r="AN14" t="inlineStr"/>
-      <c r="AO14" t="inlineStr"/>
-      <c r="AP14" t="inlineStr"/>
-      <c r="AQ14" t="inlineStr"/>
-      <c r="AR14" t="inlineStr"/>
-      <c r="AS14" t="inlineStr"/>
-      <c r="AT14" t="inlineStr"/>
-      <c r="AU14" t="inlineStr"/>
-      <c r="AV14" t="inlineStr"/>
-      <c r="AW14" t="inlineStr"/>
-      <c r="AX14" t="inlineStr"/>
-      <c r="AY14" t="inlineStr"/>
-      <c r="AZ14" t="inlineStr"/>
-      <c r="BA14" t="inlineStr"/>
       <c r="BB14" t="inlineStr">
         <is>
           <t>messenger_bag_type, non_english:aspect_Exterior Color</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>177808647882</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>LOUIS VUITTON Mylockme Chain Pochette Calfskin Black</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>USD 1569.49</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Pre-owned - Fair</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Used but in good condition, lovingly maintained.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Louis Vuitton</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>M63471</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>1</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/177808647882</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Louis Vuitton</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Messenger Bags</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Crossbody</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>Leather</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>8 in</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr"/>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>Rectangle</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr"/>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>5 in</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
+      <c r="AC15" t="inlineStr">
+        <is>
+          <t>1.2 in</t>
+        </is>
+      </c>
+      <c r="AD15" t="inlineStr"/>
+      <c r="AE15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>Lock</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>Louis Vuitton Mylockme Chain</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="AJ15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AK15" t="inlineStr">
+        <is>
+          <t>Louis Vuitton Mylockme</t>
+        </is>
+      </c>
+      <c r="AL15" t="inlineStr">
+        <is>
+          <t>M63471</t>
+        </is>
+      </c>
+      <c r="AM15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>Silver</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>21.3 in</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>Metal</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>7.5 x 5 x 1.2 inches</t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr"/>
+      <c r="AS15" t="inlineStr"/>
+      <c r="AT15" t="inlineStr"/>
+      <c r="AU15" t="inlineStr"/>
+      <c r="AV15" t="inlineStr"/>
+      <c r="AW15" t="inlineStr"/>
+      <c r="AX15" t="inlineStr"/>
+      <c r="AY15" t="inlineStr"/>
+      <c r="AZ15" t="inlineStr"/>
+      <c r="BA15" t="inlineStr"/>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>messenger_bag_type, non_english:conditionDescription</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Edit: 177831378946 - GUCCI Paddle Lock GG Supreme
</commit_message>
<xml_diff>
--- a/edited.xlsx
+++ b/edited.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB15"/>
+  <dimension ref="A1:BB16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2210,7 +2210,6 @@
           <t>USD 1569.49</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>Pre-owned - Fair</t>
@@ -2241,7 +2240,6 @@
           <t>M63471</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>1</v>
       </c>
@@ -2285,32 +2283,26 @@
           <t>Leather</t>
         </is>
       </c>
-      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr">
         <is>
           <t>8 in</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr">
         <is>
           <t>Rectangle</t>
         </is>
       </c>
-      <c r="Y15" t="inlineStr"/>
       <c r="Z15" t="inlineStr">
         <is>
           <t>5 in</t>
         </is>
       </c>
-      <c r="AA15" t="inlineStr"/>
-      <c r="AB15" t="inlineStr"/>
       <c r="AC15" t="inlineStr">
         <is>
           <t>1.2 in</t>
         </is>
       </c>
-      <c r="AD15" t="inlineStr"/>
       <c r="AE15" t="inlineStr">
         <is>
           <t>No</t>
@@ -2326,7 +2318,6 @@
           <t>Louis Vuitton Mylockme Chain</t>
         </is>
       </c>
-      <c r="AH15" t="inlineStr"/>
       <c r="AI15" t="inlineStr">
         <is>
           <t>Spain</t>
@@ -2372,19 +2363,147 @@
           <t>7.5 x 5 x 1.2 inches</t>
         </is>
       </c>
-      <c r="AR15" t="inlineStr"/>
-      <c r="AS15" t="inlineStr"/>
-      <c r="AT15" t="inlineStr"/>
-      <c r="AU15" t="inlineStr"/>
-      <c r="AV15" t="inlineStr"/>
-      <c r="AW15" t="inlineStr"/>
-      <c r="AX15" t="inlineStr"/>
-      <c r="AY15" t="inlineStr"/>
-      <c r="AZ15" t="inlineStr"/>
-      <c r="BA15" t="inlineStr"/>
       <c r="BB15" t="inlineStr">
         <is>
           <t>messenger_bag_type, non_english:conditionDescription</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>177831378946</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>GUCCI Paddle Lock GG Supreme Canvas Shoulder Bag Small 811705</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>USD 1064.91</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Pre-owned - Good</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Some signs of use, but well-maintained and in good condition</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>811705</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/177831378946</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Shoulder Bag</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Multicolor</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Leather</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Gucci GG</t>
+        </is>
+      </c>
+      <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
+      <c r="Z16" t="inlineStr"/>
+      <c r="AA16" t="inlineStr"/>
+      <c r="AB16" t="inlineStr"/>
+      <c r="AC16" t="inlineStr"/>
+      <c r="AD16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr"/>
+      <c r="AF16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr"/>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AJ16" t="inlineStr"/>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>811705</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr"/>
+      <c r="AN16" t="inlineStr"/>
+      <c r="AO16" t="inlineStr"/>
+      <c r="AP16" t="inlineStr"/>
+      <c r="AQ16" t="inlineStr"/>
+      <c r="AR16" t="inlineStr"/>
+      <c r="AS16" t="inlineStr"/>
+      <c r="AT16" t="inlineStr"/>
+      <c r="AU16" t="inlineStr"/>
+      <c r="AV16" t="inlineStr"/>
+      <c r="AW16" t="inlineStr"/>
+      <c r="AX16" t="inlineStr"/>
+      <c r="AY16" t="inlineStr"/>
+      <c r="AZ16" t="inlineStr"/>
+      <c r="BA16" t="inlineStr"/>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>messenger_bag_type, non_english:description</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Edit: 178045045305 - GUCCI Opidia GG Crossback Mini
</commit_message>
<xml_diff>
--- a/edited.xlsx
+++ b/edited.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB16"/>
+  <dimension ref="A1:BB17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2385,7 +2385,6 @@
           <t>USD 1064.91</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>Pre-owned - Good</t>
@@ -2416,7 +2415,6 @@
           <t>811705</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="n">
         <v>1</v>
       </c>
@@ -2440,7 +2438,6 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr">
         <is>
           <t>Shoulder Bag</t>
@@ -2456,54 +2453,166 @@
           <t>Leather</t>
         </is>
       </c>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr">
         <is>
           <t>Gucci GG</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
-      <c r="AA16" t="inlineStr"/>
-      <c r="AB16" t="inlineStr"/>
-      <c r="AC16" t="inlineStr"/>
-      <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="inlineStr"/>
-      <c r="AF16" t="inlineStr"/>
-      <c r="AG16" t="inlineStr"/>
-      <c r="AH16" t="inlineStr"/>
       <c r="AI16" t="inlineStr">
         <is>
           <t>Italy</t>
         </is>
       </c>
-      <c r="AJ16" t="inlineStr"/>
-      <c r="AK16" t="inlineStr"/>
       <c r="AL16" t="inlineStr">
         <is>
           <t>811705</t>
         </is>
       </c>
-      <c r="AM16" t="inlineStr"/>
-      <c r="AN16" t="inlineStr"/>
-      <c r="AO16" t="inlineStr"/>
-      <c r="AP16" t="inlineStr"/>
-      <c r="AQ16" t="inlineStr"/>
-      <c r="AR16" t="inlineStr"/>
-      <c r="AS16" t="inlineStr"/>
-      <c r="AT16" t="inlineStr"/>
-      <c r="AU16" t="inlineStr"/>
-      <c r="AV16" t="inlineStr"/>
-      <c r="AW16" t="inlineStr"/>
-      <c r="AX16" t="inlineStr"/>
-      <c r="AY16" t="inlineStr"/>
-      <c r="AZ16" t="inlineStr"/>
-      <c r="BA16" t="inlineStr"/>
       <c r="BB16" t="inlineStr">
         <is>
           <t>messenger_bag_type, non_english:description</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>178045045305</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>GUCCI Opidia GG Crossback Mini 723619</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>USD 610.91</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Pre-owned - Good</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Some signs of use, but well-maintained and in good condition.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>723619</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178045045305</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Shoulder Bag</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Gucci GG</t>
+        </is>
+      </c>
+      <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
+      <c r="Z17" t="inlineStr"/>
+      <c r="AA17" t="inlineStr"/>
+      <c r="AB17" t="inlineStr"/>
+      <c r="AC17" t="inlineStr"/>
+      <c r="AD17" t="inlineStr"/>
+      <c r="AE17" t="inlineStr"/>
+      <c r="AF17" t="inlineStr"/>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>Opidia</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr">
+        <is>
+          <t>723619</t>
+        </is>
+      </c>
+      <c r="AM17" t="inlineStr"/>
+      <c r="AN17" t="inlineStr"/>
+      <c r="AO17" t="inlineStr"/>
+      <c r="AP17" t="inlineStr"/>
+      <c r="AQ17" t="inlineStr"/>
+      <c r="AR17" t="inlineStr"/>
+      <c r="AS17" t="inlineStr"/>
+      <c r="AT17" t="inlineStr"/>
+      <c r="AU17" t="inlineStr"/>
+      <c r="AV17" t="inlineStr"/>
+      <c r="AW17" t="inlineStr"/>
+      <c r="AX17" t="inlineStr"/>
+      <c r="AY17" t="inlineStr"/>
+      <c r="AZ17" t="inlineStr"/>
+      <c r="BA17" t="inlineStr"/>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>messenger_bag_type</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Edit: 178036747772 - GUCCI Jackie 1961 Shoulder Bag Small
</commit_message>
<xml_diff>
--- a/edited.xlsx
+++ b/edited.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BB17"/>
+  <dimension ref="A1:BB18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2490,7 +2490,6 @@
           <t>USD 610.91</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>Pre-owned - Good</t>
@@ -2521,7 +2520,6 @@
           <t>723619</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
         <v>1</v>
       </c>
@@ -2545,7 +2543,6 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr">
         <is>
           <t>Shoulder Bag</t>
@@ -2561,58 +2558,171 @@
           <t>PVC</t>
         </is>
       </c>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr">
         <is>
           <t>Gucci GG</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="inlineStr"/>
-      <c r="AB17" t="inlineStr"/>
-      <c r="AC17" t="inlineStr"/>
-      <c r="AD17" t="inlineStr"/>
-      <c r="AE17" t="inlineStr"/>
-      <c r="AF17" t="inlineStr"/>
       <c r="AG17" t="inlineStr">
         <is>
           <t>Opidia</t>
         </is>
       </c>
-      <c r="AH17" t="inlineStr"/>
       <c r="AI17" t="inlineStr">
         <is>
           <t>Italy</t>
         </is>
       </c>
-      <c r="AJ17" t="inlineStr"/>
-      <c r="AK17" t="inlineStr"/>
       <c r="AL17" t="inlineStr">
         <is>
           <t>723619</t>
         </is>
       </c>
-      <c r="AM17" t="inlineStr"/>
-      <c r="AN17" t="inlineStr"/>
-      <c r="AO17" t="inlineStr"/>
-      <c r="AP17" t="inlineStr"/>
-      <c r="AQ17" t="inlineStr"/>
-      <c r="AR17" t="inlineStr"/>
-      <c r="AS17" t="inlineStr"/>
-      <c r="AT17" t="inlineStr"/>
-      <c r="AU17" t="inlineStr"/>
-      <c r="AV17" t="inlineStr"/>
-      <c r="AW17" t="inlineStr"/>
-      <c r="AX17" t="inlineStr"/>
-      <c r="AY17" t="inlineStr"/>
-      <c r="AZ17" t="inlineStr"/>
-      <c r="BA17" t="inlineStr"/>
       <c r="BB17" t="inlineStr">
         <is>
           <t>messenger_bag_type</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>178036747772</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>GUCCI Jackie 1961 Shoulder Bag Small 636706</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>USD 1189.10</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Pre-owned - Good</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Minimal signs of use, can be enjoyed as if it were new.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>169291</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Clothing, Shoes &amp; Accessories|Women|Women's Bags &amp; Handbags</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>636706</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>sazo_global</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>https://www.ebay.com/itm/178036747772</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Gucci</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Shoulder Bag</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Multicolor</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>Canvas</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
+      <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
+      <c r="Z18" t="inlineStr"/>
+      <c r="AA18" t="inlineStr"/>
+      <c r="AB18" t="inlineStr"/>
+      <c r="AC18" t="inlineStr"/>
+      <c r="AD18" t="inlineStr"/>
+      <c r="AE18" t="inlineStr"/>
+      <c r="AF18" t="inlineStr"/>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>GUCCI Jackie</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr">
+        <is>
+          <t>Gucci Jackie 1961</t>
+        </is>
+      </c>
+      <c r="AL18" t="inlineStr">
+        <is>
+          <t>636706</t>
+        </is>
+      </c>
+      <c r="AM18" t="inlineStr"/>
+      <c r="AN18" t="inlineStr"/>
+      <c r="AO18" t="inlineStr"/>
+      <c r="AP18" t="inlineStr"/>
+      <c r="AQ18" t="inlineStr"/>
+      <c r="AR18" t="inlineStr"/>
+      <c r="AS18" t="inlineStr"/>
+      <c r="AT18" t="inlineStr"/>
+      <c r="AU18" t="inlineStr"/>
+      <c r="AV18" t="inlineStr"/>
+      <c r="AW18" t="inlineStr"/>
+      <c r="AX18" t="inlineStr"/>
+      <c r="AY18" t="inlineStr"/>
+      <c r="AZ18" t="inlineStr"/>
+      <c r="BA18" t="inlineStr"/>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>messenger_bag_type, non_english:description</t>
         </is>
       </c>
     </row>

</xml_diff>